<commit_message>
build: exclude sql backup helper from electron package and update test exports
</commit_message>
<xml_diff>
--- a/test-exports/customer-ledger-2020-01-01-to-2030-01-01.xlsx
+++ b/test-exports/customer-ledger-2020-01-01-to-2030-01-01.xlsx
@@ -6,25 +6,34 @@
   <sheets>
     <sheet sheetId="1" name="Customer ledger" state="visible" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Customer ledger'!$6:$6</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="54">
   <si>
     <t>Customer Ledger</t>
   </si>
   <si>
-    <t>2020-01-01 to 2030-01-01 | 9 entries</t>
-  </si>
-  <si>
-    <t>Credit issued</t>
+    <t>01-01-2020 to 01-01-2030 (India Standard Time) | 15 entries</t>
+  </si>
+  <si>
+    <t>Opening due</t>
+  </si>
+  <si>
+    <t>Due added</t>
   </si>
   <si>
     <t>Payments received</t>
   </si>
   <si>
+    <t>Closing due</t>
+  </si>
+  <si>
     <t>Ledger entries</t>
   </si>
   <si>
@@ -43,7 +52,19 @@
     <t>Invoice no.</t>
   </si>
   <si>
-    <t>Amount</t>
+    <t>Due / debit</t>
+  </si>
+  <si>
+    <t>Payment / credit</t>
+  </si>
+  <si>
+    <t>Ledger change</t>
+  </si>
+  <si>
+    <t>Running due</t>
+  </si>
+  <si>
+    <t>Payment method</t>
   </si>
   <si>
     <t>Reference</t>
@@ -52,7 +73,9 @@
     <t>Note</t>
   </si>
   <si>
-    <t>9529138839</t>
+    <r>
+      <t>9529138839</t>
+    </r>
   </si>
   <si>
     <t>BRUCE</t>
@@ -61,79 +84,136 @@
     <t>Sale credit (due)</t>
   </si>
   <si>
-    <t>INV-20260821-57724</t>
+    <r>
+      <t>INV-20260821-57724</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from INV-20260821-57724</t>
   </si>
   <si>
-    <t>9423232371</t>
+    <r>
+      <t>9423232371</t>
+    </r>
   </si>
   <si>
     <t>Kalyan Abuj</t>
   </si>
   <si>
-    <t>INV-20260821-99852</t>
+    <r>
+      <t>INV-20260821-99852</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from INV-20260821-99852</t>
   </si>
   <si>
-    <t>INV-20260821-50662</t>
+    <r>
+      <t>INV-20260821-50662</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from INV-20260821-50662</t>
   </si>
   <si>
-    <t>INV-20260821-50043</t>
+    <r>
+      <t>INV-20260821-50043</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from INV-20260821-50043</t>
   </si>
   <si>
-    <t>INV-20260823-MT5TDACR-78D3410E</t>
+    <r>
+      <t>INV-20260823-MT5TDACR-78D3410E</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from INV-20260823-MT5TDACR-78D3410E</t>
   </si>
   <si>
-    <t>202608270009</t>
+    <r>
+      <t>202608270009</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from 202608270009</t>
   </si>
   <si>
-    <t>9848355987</t>
+    <r>
+      <t>9848355987</t>
+    </r>
   </si>
   <si>
     <t>Deep Audit Customer</t>
   </si>
   <si>
-    <t>INV-AUDIT-5992</t>
+    <r>
+      <t>INV-AUDIT-5992</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from INV-AUDIT-5992</t>
   </si>
   <si>
-    <t>202608280001</t>
+    <r>
+      <t>202608280001</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from 202608280001</t>
   </si>
   <si>
-    <t>202608280004</t>
+    <r>
+      <t>202608280004</t>
+    </r>
   </si>
   <si>
     <t>Credit balance from 202608280004</t>
+  </si>
+  <si>
+    <t>Payment received</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <r>
+      <t>RCPT-7189116</t>
+    </r>
+  </si>
+  <si>
+    <t>Payment received against INV-20260821-57724</t>
+  </si>
+  <si>
+    <t>Payment received against INV-20260821-50662</t>
+  </si>
+  <si>
+    <t>Payment received against INV-20260821-50043</t>
+  </si>
+  <si>
+    <t>Payment received against INV-20260823-MT5TDACR-78D3410E</t>
+  </si>
+  <si>
+    <t>Payment received against 202608280004</t>
+  </si>
+  <si>
+    <r>
+      <t>202608280017</t>
+    </r>
+  </si>
+  <si>
+    <t>Credit balance from 202608280017</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="[$₹-en-IN]#,##0.00;[Red]-[$₹-en-IN]#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="#,##0;[Red]-#,##0"/>
+    <numFmt numFmtId="166" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -168,7 +248,7 @@
       <color rgb="FF271A05"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -193,6 +273,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD5A044"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFCF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -220,9 +310,15 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="thin">
+        <color rgb="FFE8E1D8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE8E1D8"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE8E1D8"/>
+      </top>
       <bottom style="thin">
         <color rgb="FFE8E1D8"/>
       </bottom>
@@ -232,31 +328,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -277,8 +388,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="KusumExport1" displayName="KusumExport1" ref="A5:H14" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A5:H14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="KusumExport1" displayName="KusumExport1" ref="A6:M21" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A6:M21">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -287,18 +398,28 @@
     <filterColumn colId="5" hiddenButton="1"/>
     <filterColumn colId="6" hiddenButton="1"/>
     <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="8">
+  <tableColumns count="13">
     <tableColumn id="1" name="Ledger date" totalsRowLabel="Total"/>
     <tableColumn id="2" name="Phone / ID" totalsRowFunction="none"/>
     <tableColumn id="3" name="Customer" totalsRowFunction="none"/>
     <tableColumn id="4" name="Entry type" totalsRowFunction="none"/>
     <tableColumn id="5" name="Invoice no." totalsRowFunction="none"/>
-    <tableColumn id="6" name="Amount" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Reference" totalsRowFunction="none"/>
-    <tableColumn id="8" name="Note" totalsRowFunction="none"/>
+    <tableColumn id="6" name="Due / debit" totalsRowFunction="none"/>
+    <tableColumn id="7" name="Payment / credit" totalsRowFunction="none"/>
+    <tableColumn id="8" name="Ledger change" totalsRowFunction="none"/>
+    <tableColumn id="9" name="Opening due" totalsRowFunction="none"/>
+    <tableColumn id="10" name="Running due" totalsRowFunction="none"/>
+    <tableColumn id="11" name="Payment method" totalsRowFunction="none"/>
+    <tableColumn id="12" name="Reference" totalsRowFunction="none"/>
+    <tableColumn id="13" name="Note" totalsRowFunction="none"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -627,20 +748,21 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="6" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -651,8 +773,13 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -663,294 +790,714 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4">
-        <v>162237.63999999998</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="4">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3"/>
+      <c r="G3" s="4">
+        <v>169808.13999999998</v>
+      </c>
+      <c r="H3" s="4"/>
+      <c r="I3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="5">
+      <c r="J3" s="3"/>
+      <c r="K3" s="4">
+        <v>69779.33</v>
+      </c>
+      <c r="L3" s="4"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="4">
+        <v>100028.81</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="5">
+        <v>15</v>
+      </c>
+      <c r="H4" s="5"/>
+    </row>
+    <row r="6" ht="26" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
-        <v>46246.94666666667</v>
-      </c>
-      <c r="B6" s="8" t="s">
+      <c r="G6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="H6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="I6" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="K6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="9">
+      <c r="L6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>46247.5</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="10">
         <v>205</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
-        <v>46247.43103009259</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="8" t="s">
+      <c r="G7" s="10">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10">
+        <v>205</v>
+      </c>
+      <c r="I7" s="10">
+        <v>0</v>
+      </c>
+      <c r="J7" s="10">
+        <v>205</v>
+      </c>
+      <c r="K7" s="9"/>
+      <c r="L7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="11">
+        <v>46247.5</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="14">
+        <v>11896.5</v>
+      </c>
+      <c r="G8" s="14">
+        <v>0</v>
+      </c>
+      <c r="H8" s="14">
+        <v>11896.5</v>
+      </c>
+      <c r="I8" s="14">
+        <v>0</v>
+      </c>
+      <c r="J8" s="14">
+        <v>11896.5</v>
+      </c>
+      <c r="K8" s="13"/>
+      <c r="L8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="M8" s="13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="7">
+        <v>46247.5</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="9">
-        <v>11896.5</v>
-      </c>
-      <c r="G7" s="8" t="s">
+      <c r="D9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="10">
+        <v>28724.64</v>
+      </c>
+      <c r="G9" s="10">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10">
+        <v>28724.64</v>
+      </c>
+      <c r="I9" s="10">
+        <v>0</v>
+      </c>
+      <c r="J9" s="10">
+        <v>28929.64</v>
+      </c>
+      <c r="K9" s="9"/>
+      <c r="L9" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="M9" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="11">
+        <v>46247.5</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="D10" s="13" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
-        <v>46247.44598379629</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="8" t="s">
+      <c r="E10" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="14">
+        <v>40553.16</v>
+      </c>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+      <c r="H10" s="14">
+        <v>40553.16</v>
+      </c>
+      <c r="I10" s="14">
+        <v>0</v>
+      </c>
+      <c r="J10" s="14">
+        <v>69482.8</v>
+      </c>
+      <c r="K10" s="13"/>
+      <c r="L10" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M10" s="13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="7">
+        <v>46249.5</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="10">
+        <v>296.5</v>
+      </c>
+      <c r="G11" s="10">
+        <v>0</v>
+      </c>
+      <c r="H11" s="10">
+        <v>296.5</v>
+      </c>
+      <c r="I11" s="10">
+        <v>0</v>
+      </c>
+      <c r="J11" s="10">
+        <v>69779.3</v>
+      </c>
+      <c r="K11" s="9"/>
+      <c r="L11" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M11" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="11">
+        <v>46259.5</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0.28</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>0.28</v>
+      </c>
+      <c r="I12" s="14">
+        <v>0</v>
+      </c>
+      <c r="J12" s="14">
+        <v>11896.78</v>
+      </c>
+      <c r="K12" s="13"/>
+      <c r="L12" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="M12" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="7">
+        <v>46260.5</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="10">
+        <v>80561.48</v>
+      </c>
+      <c r="G13" s="10">
+        <v>0</v>
+      </c>
+      <c r="H13" s="10">
+        <v>80561.48</v>
+      </c>
+      <c r="I13" s="10">
+        <v>0</v>
+      </c>
+      <c r="J13" s="10">
+        <v>80561.48</v>
+      </c>
+      <c r="K13" s="9"/>
+      <c r="L13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="M13" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="11">
+        <v>46262.5</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="14">
+        <v>0.05</v>
+      </c>
+      <c r="G14" s="14">
+        <v>0</v>
+      </c>
+      <c r="H14" s="14">
+        <v>0.05</v>
+      </c>
+      <c r="I14" s="14">
+        <v>0</v>
+      </c>
+      <c r="J14" s="14">
+        <v>11896.83</v>
+      </c>
+      <c r="K14" s="13"/>
+      <c r="L14" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="M14" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="7">
+        <v>46262.5</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="10">
+        <v>0.03</v>
+      </c>
+      <c r="G15" s="10">
+        <v>0</v>
+      </c>
+      <c r="H15" s="10">
+        <v>0.03</v>
+      </c>
+      <c r="I15" s="10">
+        <v>0</v>
+      </c>
+      <c r="J15" s="10">
+        <v>69779.33</v>
+      </c>
+      <c r="K15" s="9"/>
+      <c r="L15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="M15" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="11">
+        <v>46262.5</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F16" s="14">
+        <v>0</v>
+      </c>
+      <c r="G16" s="14">
+        <v>205</v>
+      </c>
+      <c r="H16" s="14">
+        <v>-205</v>
+      </c>
+      <c r="I16" s="14">
+        <v>0</v>
+      </c>
+      <c r="J16" s="14">
+        <v>69574.33</v>
+      </c>
+      <c r="K16" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="L16" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="M16" s="13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="7">
+        <v>46262.5</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="10">
+        <v>0</v>
+      </c>
+      <c r="G17" s="10">
         <v>28724.64</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
-        <v>46247.45211805556</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="9">
+      <c r="H17" s="10">
+        <v>-28724.64</v>
+      </c>
+      <c r="I17" s="10">
+        <v>0</v>
+      </c>
+      <c r="J17" s="10">
+        <v>40849.69</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="M17" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="11">
+        <v>46262.5</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
         <v>40553.16</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
-        <v>46249.29170138889</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="9">
+      <c r="H18" s="14">
+        <v>-40553.16</v>
+      </c>
+      <c r="I18" s="14">
+        <v>0</v>
+      </c>
+      <c r="J18" s="14">
+        <v>296.52999999999884</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="L18" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="M18" s="13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="7">
+        <v>46262.5</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="10">
+        <v>0</v>
+      </c>
+      <c r="G19" s="10">
         <v>296.5</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
-        <v>46259.383831018524</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="8" t="s">
+      <c r="H19" s="10">
+        <v>-296.5</v>
+      </c>
+      <c r="I19" s="10">
+        <v>0</v>
+      </c>
+      <c r="J19" s="10">
+        <v>0.029999999998835847</v>
+      </c>
+      <c r="K19" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="M19" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="11">
+        <v>46262.5</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="9">
-        <v>0.28</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
-        <v>46260.085138888884</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="9">
-        <v>80561.48</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="7">
-        <v>46261.81839</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="8" t="s">
+      <c r="C20" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="14">
+        <v>0</v>
+      </c>
+      <c r="G20" s="14">
+        <v>0.03</v>
+      </c>
+      <c r="H20" s="14">
+        <v>-0.03</v>
+      </c>
+      <c r="I20" s="14">
+        <v>0</v>
+      </c>
+      <c r="J20" s="14">
+        <v>-1.1641521080463235e-12</v>
+      </c>
+      <c r="K20" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="L20" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="M20" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="7">
+        <v>46262.5</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F13" s="9">
-        <v>0.05</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
-        <v>46261.836441203704</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="F14" s="9">
-        <v>0.03</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>37</v>
+      <c r="C21" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F21" s="10">
+        <v>7570.5</v>
+      </c>
+      <c r="G21" s="10">
+        <v>0</v>
+      </c>
+      <c r="H21" s="10">
+        <v>7570.5</v>
+      </c>
+      <c r="I21" s="10">
+        <v>0</v>
+      </c>
+      <c r="J21" s="10">
+        <v>7570.499999999999</v>
+      </c>
+      <c r="K21" s="9"/>
+      <c r="L21" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="M21" s="9" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H14"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
+  <autoFilter ref="A6:M21"/>
+  <mergeCells count="12">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
   </mergeCells>
-  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</evenFooter>
+  </headerFooter>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>